<commit_message>
Add release/8.0.12 to meta-sheet
</commit_message>
<xml_diff>
--- a/meta-sheet.xlsx
+++ b/meta-sheet.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.005" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -806,6 +806,33 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>release/8.0.12</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>